<commit_message>
Revise all notebooks for WT 2026/27
- Fix errors found in the audit: Session 2 merge labels, UTC times and
  NameError; Session 6 GAM evaluated on the test set; Session 7 lasso
  that was ridge, in-sample meta-learner and RocCurveDisplay crash;
  Session 10 unbatched training; Session 12 PDP crash on integer columns
  and permutation importance on training data; and more
- Align terminology and notation with ISLP and reference the matching
  chapters, sections and labs under each notebook title
- Harmonize layout (Initialize notebook, Problem description, Load data,
  Prepare data, ..., Your turn!), strip outputs, use the python3 kernel
- Add explanations and clear exercise prompts; exercise cells are empty
- Load all data from ds4b-2026; remove global warning suppression
- Remove redundant micromortgage_stacking.ipynb; update README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Session_03/gradient_descent.xlsx
+++ b/Session_03/gradient_descent.xlsx
@@ -13,8 +13,8 @@
     <workbookView xWindow="45040" yWindow="-1820" windowWidth="30240" windowHeight="17260" xr2:uid="{63849087-0FE2-AF4B-ACB7-CB07C279593B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Gradient Desent" sheetId="1" r:id="rId1"/>
-    <sheet name="Gradient Desent (solved)" sheetId="2" r:id="rId2"/>
+    <sheet name="Gradient Descent" sheetId="1" r:id="rId1"/>
+    <sheet name="Gradient Descent (solved)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>